<commit_message>
Remove prototype wording from Trend Research reports
</commit_message>
<xml_diff>
--- a/jamify_results.xlsx
+++ b/jamify_results.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trend Research" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Trend Research" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -468,7 +468,7 @@
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>Pain Points</t>
+          <t>Check Before Buying</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
@@ -518,7 +518,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Review scan not wired yet</t>
+          <t>Check current reviews, shipping cost, return risk, and seller pricing before buying inventory.</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -568,7 +568,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Review scan not wired yet</t>
+          <t>Check current reviews, shipping cost, return risk, and seller pricing before buying inventory.</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">

</xml_diff>